<commit_message>
brainAGE permutation and bootstrapping method and qq-plots generated.
</commit_message>
<xml_diff>
--- a/analyses/brainage_gap/outputs/permutation/two_sample_permutation_summary.xlsx
+++ b/analyses/brainage_gap/outputs/permutation/two_sample_permutation_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,55 +446,60 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>N_Test</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>N_Ref</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Test_MAE</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Ref_MAE</t>
+          <t>Test_Mean</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Observed_Delta_MAE</t>
+          <t>Ref_Mean</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Observed_Delta</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Null_Mean_Delta</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Null_95_Lower</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Null_95_Upper</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>p_value_error_increase</t>
-        </is>
-      </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>p_value_greater</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>p_value_two_sided</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Plot_Path</t>
         </is>
@@ -503,7 +508,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Chinese</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -516,46 +521,51 @@
           <t>40-90</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>326</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E2" t="n">
+        <v>159</v>
+      </c>
+      <c r="F2" t="n">
         <v>9493</v>
       </c>
-      <c r="F2" t="n">
-        <v>3.878086577778324</v>
-      </c>
       <c r="G2" t="n">
-        <v>3.083662273838618</v>
+        <v>1.363774017757769</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7944243039397061</v>
+        <v>0.01420426200463499</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.002416183792107716</v>
+        <v>1.349569755753134</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.268992414270358</v>
+        <v>0.003968698839948851</v>
       </c>
       <c r="K2" t="n">
-        <v>0.271279074063892</v>
+        <v>-0.6062329724940398</v>
       </c>
       <c r="L2" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.6227694072985385</v>
       </c>
       <c r="M2" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Female_40-90_permutation_histogram.png</t>
+      <c r="N2" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Black/Black_Female_40-90_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chinese</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -565,49 +575,54 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>5-40</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>547</v>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>8505</v>
+        <v>159</v>
       </c>
       <c r="F3" t="n">
-        <v>2.988168294188121</v>
+        <v>9493</v>
       </c>
       <c r="G3" t="n">
-        <v>1.448046302578601</v>
+        <v>3.20139752215051</v>
       </c>
       <c r="H3" t="n">
-        <v>1.54012199160952</v>
+        <v>3.083662273838618</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.0004681631860056226</v>
+        <v>0.1177352483118925</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.1104998567359042</v>
+        <v>0.001954418892464116</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1142892358472945</v>
+        <v>-0.3605321192761762</v>
       </c>
       <c r="L3" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.3817355263697571</v>
       </c>
       <c r="M3" t="n">
-        <v>9.999000099990002e-05</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Female_5-40_permutation_histogram.png</t>
+        <v>0.2692730726927307</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.5378462153784621</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Black/Black_Female_40-90_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Chinese</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -620,46 +635,51 @@
           <t>40-90</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>198</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E4" t="n">
+        <v>125</v>
+      </c>
+      <c r="F4" t="n">
         <v>7788</v>
       </c>
-      <c r="F4" t="n">
-        <v>3.879296074389766</v>
-      </c>
       <c r="G4" t="n">
-        <v>3.229780626449666</v>
+        <v>2.44134560861103</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6495154479401002</v>
+        <v>-0.008569098016178771</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.0003734802931437632</v>
+        <v>2.449914706627208</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.3453155771371014</v>
+        <v>0.004353845949406358</v>
       </c>
       <c r="K4" t="n">
-        <v>0.3614581168619875</v>
+        <v>-0.7277096722586702</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0001999800019998</v>
+        <v>0.7422414468243337</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0001999800019998</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Male_40-90_permutation_histogram.png</t>
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N4" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Black/Black_Male_40-90_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chinese</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -669,49 +689,54 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5-40</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>418</v>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>7541</v>
+        <v>125</v>
       </c>
       <c r="F5" t="n">
-        <v>2.81899004980348</v>
+        <v>7788</v>
       </c>
       <c r="G5" t="n">
-        <v>1.496159184830526</v>
+        <v>3.839051567340491</v>
       </c>
       <c r="H5" t="n">
-        <v>1.322830864972953</v>
+        <v>3.229780626449666</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.0007427212736076194</v>
+        <v>0.6092709408908257</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.1229927517934886</v>
+        <v>-0.0004737999228550743</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1286201887128629</v>
+        <v>-0.4259244250024591</v>
       </c>
       <c r="L5" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.4540637250901876</v>
       </c>
       <c r="M5" t="n">
-        <v>9.999000099990002e-05</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Male_5-40_permutation_histogram.png</t>
+        <v>0.0045995400459954</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.0071992800719928</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Black/Black_Male_40-90_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Chilean</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -721,49 +746,54 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>40-90</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>187</v>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>9493</v>
+        <v>27</v>
       </c>
       <c r="F6" t="n">
-        <v>4.562076869862906</v>
+        <v>8505</v>
       </c>
       <c r="G6" t="n">
-        <v>3.083662273838618</v>
+        <v>3.44301259731997</v>
       </c>
       <c r="H6" t="n">
-        <v>1.478414596024288</v>
+        <v>-0.008381465306172826</v>
       </c>
       <c r="I6" t="n">
-        <v>0.002010053971126692</v>
+        <v>3.451394062626143</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.3436989682825571</v>
+        <v>-0.005498181466366416</v>
       </c>
       <c r="K6" t="n">
-        <v>0.3540557958788425</v>
+        <v>-0.7064892462504806</v>
       </c>
       <c r="L6" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.7284773628393884</v>
       </c>
       <c r="M6" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Female_40-90_permutation_histogram.png</t>
+      <c r="N6" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chilean/Chilean_Female_5-40_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Chilean</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -776,46 +806,51 @@
           <t>5-40</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>216</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F7" t="n">
         <v>8505</v>
       </c>
-      <c r="F7" t="n">
-        <v>2.550990304857664</v>
-      </c>
       <c r="G7" t="n">
+        <v>3.527012956891982</v>
+      </c>
+      <c r="H7" t="n">
         <v>1.448046302578601</v>
       </c>
-      <c r="H7" t="n">
-        <v>1.102944002279063</v>
-      </c>
       <c r="I7" t="n">
-        <v>0.0005857294504767028</v>
+        <v>2.078966654313381</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.1560461235580151</v>
+        <v>0.001014929571725401</v>
       </c>
       <c r="K7" t="n">
-        <v>0.168166504289291</v>
+        <v>-0.4049429383527437</v>
       </c>
       <c r="L7" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.4849944640637287</v>
       </c>
       <c r="M7" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Female_5-40_permutation_histogram.png</t>
+      <c r="N7" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chilean/Chilean_Female_5-40_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Chilean</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -825,49 +860,54 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>40-90</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>128</v>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E8" t="n">
-        <v>7788</v>
+        <v>56</v>
       </c>
       <c r="F8" t="n">
-        <v>4.367684813770984</v>
+        <v>7541</v>
       </c>
       <c r="G8" t="n">
-        <v>3.229780626449666</v>
+        <v>2.08361888900311</v>
       </c>
       <c r="H8" t="n">
-        <v>1.137904187321318</v>
+        <v>-0.003283886222118988</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.003935682660968116</v>
+        <v>2.086902775225229</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.4291832222008403</v>
+        <v>0.004487753457367792</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4422492654819042</v>
+        <v>-0.489568925177703</v>
       </c>
       <c r="L8" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.5114201559175816</v>
       </c>
       <c r="M8" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Male_40-90_permutation_histogram.png</t>
+      <c r="N8" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chilean/Chilean_Male_5-40_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Chilean</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -880,46 +920,51 @@
           <t>5-40</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>389</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F9" t="n">
         <v>7541</v>
       </c>
-      <c r="F9" t="n">
-        <v>2.814730357072431</v>
-      </c>
       <c r="G9" t="n">
+        <v>3.395465014111248</v>
+      </c>
+      <c r="H9" t="n">
         <v>1.496159184830526</v>
       </c>
-      <c r="H9" t="n">
-        <v>1.318571172241904</v>
-      </c>
       <c r="I9" t="n">
-        <v>-0.0006533121226252828</v>
+        <v>1.899305829280722</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.1264436659836633</v>
+        <v>-0.001830669545082886</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1334036251461429</v>
+        <v>-0.2923187357660768</v>
       </c>
       <c r="L9" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.3314357184626717</v>
       </c>
       <c r="M9" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Male_5-40_permutation_histogram.png</t>
+      <c r="N9" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chilean/Chilean_Male_5-40_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mexican</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -932,46 +977,51 @@
           <t>40-90</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>31</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E10" t="n">
+        <v>324</v>
+      </c>
+      <c r="F10" t="n">
         <v>9493</v>
       </c>
-      <c r="F10" t="n">
-        <v>6.497673760343709</v>
-      </c>
       <c r="G10" t="n">
-        <v>3.083662273838618</v>
+        <v>2.432773870383416</v>
       </c>
       <c r="H10" t="n">
-        <v>3.414011486505091</v>
+        <v>0.01420426200463499</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.002045206655360105</v>
+        <v>2.41856960837878</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.8046241776849642</v>
+        <v>-0.003643683265344916</v>
       </c>
       <c r="K10" t="n">
-        <v>0.9010249687268741</v>
+        <v>-0.4378051573596786</v>
       </c>
       <c r="L10" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.4408604065767088</v>
       </c>
       <c r="M10" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Female_40-90_permutation_histogram.png</t>
+      <c r="N10" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Female_40-90_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mexican</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -981,106 +1031,116 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5-40</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>106</v>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E11" t="n">
-        <v>8505</v>
+        <v>324</v>
       </c>
       <c r="F11" t="n">
-        <v>2.876220872815426</v>
+        <v>9493</v>
       </c>
       <c r="G11" t="n">
-        <v>1.448046302578601</v>
+        <v>3.891747656538398</v>
       </c>
       <c r="H11" t="n">
-        <v>1.428174570236825</v>
+        <v>3.083662273838618</v>
       </c>
       <c r="I11" t="n">
-        <v>7.977190393906373e-05</v>
+        <v>0.8080853826997805</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.2133062268565359</v>
+        <v>0.001318875985636835</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2363939108170568</v>
+        <v>-0.2591504941258182</v>
       </c>
       <c r="L11" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.2732179211243828</v>
       </c>
       <c r="M11" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Female_5-40_permutation_histogram.png</t>
+      <c r="N11" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Female_40-90_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mexican</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>40-90</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>13</v>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E12" t="n">
-        <v>7788</v>
+        <v>547</v>
       </c>
       <c r="F12" t="n">
-        <v>3.232578982110632</v>
+        <v>8505</v>
       </c>
       <c r="G12" t="n">
-        <v>3.229780626449666</v>
+        <v>2.167043180506354</v>
       </c>
       <c r="H12" t="n">
-        <v>0.002798355660965868</v>
+        <v>-0.008381465306172826</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.004725498239706341</v>
+        <v>2.175424645812527</v>
       </c>
       <c r="J12" t="n">
-        <v>-1.255856895003357</v>
+        <v>0.001988983742005269</v>
       </c>
       <c r="K12" t="n">
-        <v>1.455311798288633</v>
+        <v>-0.1712292793572133</v>
       </c>
       <c r="L12" t="n">
-        <v>0.4726527347265274</v>
+        <v>0.17642416462809</v>
       </c>
       <c r="M12" t="n">
-        <v>0.9963003699630038</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Male_40-90_permutation_histogram.png</t>
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N12" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Female_5-40_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mexican</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1088,51 +1148,56 @@
           <t>5-40</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>164</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E13" t="n">
-        <v>7541</v>
+        <v>547</v>
       </c>
       <c r="F13" t="n">
-        <v>3.342757119408537</v>
+        <v>8505</v>
       </c>
       <c r="G13" t="n">
-        <v>1.496159184830526</v>
+        <v>2.988168294188121</v>
       </c>
       <c r="H13" t="n">
-        <v>1.84659793457801</v>
+        <v>1.448046302578601</v>
       </c>
       <c r="I13" t="n">
-        <v>0.001900866898817378</v>
+        <v>1.54012199160952</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.1818118404706433</v>
+        <v>0.0009015007134298705</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1997260224796715</v>
+        <v>-0.107641145270464</v>
       </c>
       <c r="L13" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.1153475699124295</v>
       </c>
       <c r="M13" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Male_5-40_permutation_histogram.png</t>
+      <c r="N13" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Female_5-40_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>South Asian</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1140,98 +1205,108 @@
           <t>40-90</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>144</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E14" t="n">
-        <v>9493</v>
+        <v>194</v>
       </c>
       <c r="F14" t="n">
-        <v>3.618056092100486</v>
+        <v>7788</v>
       </c>
       <c r="G14" t="n">
-        <v>3.083662273838618</v>
+        <v>2.200908610823356</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5343938182618682</v>
+        <v>-0.008569098016178771</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.0007815384572906898</v>
+        <v>2.209477708839535</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.3813857096031518</v>
+        <v>0.002015670990550653</v>
       </c>
       <c r="K14" t="n">
-        <v>0.408309293641418</v>
+        <v>-0.5834397961915948</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0044995500449955</v>
+        <v>0.5842315130275165</v>
       </c>
       <c r="M14" t="n">
-        <v>0.006799320067993201</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Female_40-90_permutation_histogram.png</t>
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N14" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Male_40-90_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>South Asian</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5-40</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>16</v>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E15" t="n">
-        <v>8505</v>
+        <v>194</v>
       </c>
       <c r="F15" t="n">
-        <v>2.177530382264464</v>
+        <v>7788</v>
       </c>
       <c r="G15" t="n">
-        <v>1.448046302578601</v>
+        <v>3.786728959590673</v>
       </c>
       <c r="H15" t="n">
-        <v>0.7294840796858637</v>
+        <v>3.229780626449666</v>
       </c>
       <c r="I15" t="n">
-        <v>0.00325915931112572</v>
+        <v>0.5569483331410074</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.5009022568564815</v>
+        <v>0.0003664496901626479</v>
       </c>
       <c r="K15" t="n">
-        <v>0.644553555077471</v>
+        <v>-0.3524591649948828</v>
       </c>
       <c r="L15" t="n">
-        <v>0.0158984101589841</v>
+        <v>0.3614069677616913</v>
       </c>
       <c r="M15" t="n">
-        <v>0.0168983101689831</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Female_5-40_permutation_histogram.png</t>
+        <v>0.0018998100189981</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.0027997200279972</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Male_40-90_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>South Asian</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1241,49 +1316,54 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>40-90</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>238</v>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E16" t="n">
-        <v>7788</v>
+        <v>418</v>
       </c>
       <c r="F16" t="n">
-        <v>3.924168775186589</v>
+        <v>7541</v>
       </c>
       <c r="G16" t="n">
-        <v>3.229780626449666</v>
+        <v>0.4370334934273646</v>
       </c>
       <c r="H16" t="n">
-        <v>0.6943881487369232</v>
+        <v>-0.003283886222118988</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.001569298435093386</v>
+        <v>0.4403173796494836</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.3176091981190896</v>
+        <v>0.0007278523004359373</v>
       </c>
       <c r="K16" t="n">
-        <v>0.3204137957296703</v>
+        <v>-0.1976743185543242</v>
       </c>
       <c r="L16" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.2036942657556868</v>
       </c>
       <c r="M16" t="n">
-        <v>0.0001999800019998</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Male_40-90_permutation_histogram.png</t>
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N16" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Male_5-40_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>South Asian</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1296,46 +1376,51 @@
           <t>5-40</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>21</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
       </c>
       <c r="E17" t="n">
+        <v>418</v>
+      </c>
+      <c r="F17" t="n">
         <v>7541</v>
       </c>
-      <c r="F17" t="n">
-        <v>2.707086686322044</v>
-      </c>
       <c r="G17" t="n">
+        <v>2.81899004980348</v>
+      </c>
+      <c r="H17" t="n">
         <v>1.496159184830526</v>
       </c>
-      <c r="H17" t="n">
-        <v>1.210927501491518</v>
-      </c>
       <c r="I17" t="n">
-        <v>0.001794962453823316</v>
+        <v>1.322830864972953</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.447748622673816</v>
+        <v>0.0004522291228042462</v>
       </c>
       <c r="K17" t="n">
-        <v>0.5510041553888674</v>
+        <v>-0.1224650679675785</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0005999400059994001</v>
+        <v>0.1297346160273337</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0005999400059994001</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Male_5-40_permutation_histogram.png</t>
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N17" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Chinese/Chinese_Male_5-40_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>Japanese</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1345,94 +1430,1586 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5-40</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>268</v>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
       </c>
       <c r="E18" t="n">
-        <v>8505</v>
+        <v>187</v>
       </c>
       <c r="F18" t="n">
-        <v>2.414725820022386</v>
+        <v>9493</v>
       </c>
       <c r="G18" t="n">
-        <v>1.448046302578601</v>
+        <v>3.377495193717641</v>
       </c>
       <c r="H18" t="n">
-        <v>0.966679517443785</v>
+        <v>0.01420426200463499</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0002608716486683523</v>
+        <v>3.363290931713006</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.1410057579742695</v>
+        <v>0.00287790742921243</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1469125174159852</v>
+        <v>-0.559777575844002</v>
       </c>
       <c r="L18" t="n">
-        <v>9.999000099990002e-05</v>
+        <v>0.560749787055545</v>
       </c>
       <c r="M18" t="n">
         <v>9.999000099990002e-05</v>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Turkish/Turkish_Female_5-40_permutation_histogram.png</t>
+      <c r="N18" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Female_40-90_BAG_permutation_histogram.png</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>187</v>
+      </c>
+      <c r="F19" t="n">
+        <v>9493</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4.562076869862906</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3.083662273838618</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.478414596024288</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-0.00122572390203074</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-0.3401293529040929</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.3533980168081154</v>
+      </c>
+      <c r="M19" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N19" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Female_40-90_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>216</v>
+      </c>
+      <c r="F20" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-1.177027639772382</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-0.008381465306172826</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-1.16864617446621</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.002672914163307929</v>
+      </c>
+      <c r="K20" t="n">
+        <v>-0.2542925638724836</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.2562463454336751</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Female_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>216</v>
+      </c>
+      <c r="F21" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2.550990304857664</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.448046302578601</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.102944002279063</v>
+      </c>
+      <c r="J21" t="n">
+        <v>-0.0003349634275595779</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-0.1572107723039188</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.1634979826689041</v>
+      </c>
+      <c r="M21" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N21" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Female_5-40_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>128</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7788</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3.239228039342565</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-0.008569098016178771</v>
+      </c>
+      <c r="I22" t="n">
+        <v>3.247797137358743</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.004786447370331538</v>
+      </c>
+      <c r="K22" t="n">
+        <v>-0.7024744442780745</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.7187741357240007</v>
+      </c>
+      <c r="M22" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N22" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Male_40-90_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>128</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7788</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4.367684813770984</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3.229780626449666</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.137904187321318</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.005301806423384105</v>
+      </c>
+      <c r="K23" t="n">
+        <v>-0.4229989543742541</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.4537828067140852</v>
+      </c>
+      <c r="M23" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N23" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Male_40-90_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>389</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7541</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-0.7710055069016482</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-0.003283886222118988</v>
+      </c>
+      <c r="I24" t="n">
+        <v>-0.7677216206795292</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.0003390068094804915</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-0.2044117471209729</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.20556001180844</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Male_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>389</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7541</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2.814730357072431</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1.496159184830526</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1.318571172241904</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.0005274543422409591</v>
+      </c>
+      <c r="K25" t="n">
+        <v>-0.1216574949447047</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.1336665578798495</v>
+      </c>
+      <c r="M25" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N25" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Japanese/Japanese_Male_5-40_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>31</v>
+      </c>
+      <c r="F26" t="n">
+        <v>9493</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6.252526153938822</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.01420426200463499</v>
+      </c>
+      <c r="I26" t="n">
+        <v>6.238321891934187</v>
+      </c>
+      <c r="J26" t="n">
+        <v>-0.003464907462694698</v>
+      </c>
+      <c r="K26" t="n">
+        <v>-1.365269342391702</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1.384850562167515</v>
+      </c>
+      <c r="M26" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N26" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Female_40-90_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>31</v>
+      </c>
+      <c r="F27" t="n">
+        <v>9493</v>
+      </c>
+      <c r="G27" t="n">
+        <v>6.497673760343709</v>
+      </c>
+      <c r="H27" t="n">
+        <v>3.083662273838618</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3.414011486505091</v>
+      </c>
+      <c r="J27" t="n">
+        <v>-0.00259512955844833</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-0.8015906102332944</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.8936434500142612</v>
+      </c>
+      <c r="M27" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N27" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Female_40-90_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>106</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-0.9768102392205783</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-0.008381465306172826</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-0.9684287739144055</v>
+      </c>
+      <c r="J28" t="n">
+        <v>-0.001461867297838836</v>
+      </c>
+      <c r="K28" t="n">
+        <v>-0.3598580923966422</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.3561912001665433</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1</v>
+      </c>
+      <c r="N28" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Female_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>106</v>
+      </c>
+      <c r="F29" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2.876220872815426</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1.448046302578601</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1.428174570236825</v>
+      </c>
+      <c r="J29" t="n">
+        <v>-0.0002281031162297509</v>
+      </c>
+      <c r="K29" t="n">
+        <v>-0.2133438158617034</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.2349837024124005</v>
+      </c>
+      <c r="M29" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N29" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Female_5-40_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>13</v>
+      </c>
+      <c r="F30" t="n">
+        <v>7788</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-0.903863382798942</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-0.008569098016178771</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-0.8952942847827632</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.01082898855998167</v>
+      </c>
+      <c r="K30" t="n">
+        <v>-2.210303475789212</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.229817681247732</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.785921407859214</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.4310568943105689</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Male_40-90_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>13</v>
+      </c>
+      <c r="F31" t="n">
+        <v>7788</v>
+      </c>
+      <c r="G31" t="n">
+        <v>3.232578982110632</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3.229780626449666</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.002798355660965868</v>
+      </c>
+      <c r="J31" t="n">
+        <v>-0.006000347576730596</v>
+      </c>
+      <c r="K31" t="n">
+        <v>-1.213936506433736</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1.438925009108952</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.4713528647135287</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.9976002399760024</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Male_40-90_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>164</v>
+      </c>
+      <c r="F32" t="n">
+        <v>7541</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-1.635154231932927</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-0.003283886222118988</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-1.631870345710808</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.002913732764321741</v>
+      </c>
+      <c r="K32" t="n">
+        <v>-0.302073020735496</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.3013809783154779</v>
+      </c>
+      <c r="M32" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Male_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Mexican</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>164</v>
+      </c>
+      <c r="F33" t="n">
+        <v>7541</v>
+      </c>
+      <c r="G33" t="n">
+        <v>3.342757119408537</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1.496159184830526</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1.84659793457801</v>
+      </c>
+      <c r="J33" t="n">
+        <v>-0.0009548661409876782</v>
+      </c>
+      <c r="K33" t="n">
+        <v>-0.1855550853354636</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.1973189139261987</v>
+      </c>
+      <c r="M33" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N33" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Mexican/Mexican_Male_5-40_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>144</v>
+      </c>
+      <c r="F34" t="n">
+        <v>9493</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2.000631904789214</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.01420426200463499</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1.98642764278458</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.000164618276883872</v>
+      </c>
+      <c r="K34" t="n">
+        <v>-0.6491350866686565</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.6457849462771804</v>
+      </c>
+      <c r="M34" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N34" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Female_40-90_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>144</v>
+      </c>
+      <c r="F35" t="n">
+        <v>9493</v>
+      </c>
+      <c r="G35" t="n">
+        <v>3.618056092100486</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3.083662273838618</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.5343938182618682</v>
+      </c>
+      <c r="J35" t="n">
+        <v>-0.00479370487872808</v>
+      </c>
+      <c r="K35" t="n">
+        <v>-0.3934631996516857</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0.4004939730518992</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.0046995300469953</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.007799220077992201</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Female_40-90_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>16</v>
+      </c>
+      <c r="F36" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-0.3181752091999246</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-0.008381465306172826</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-0.3097937438937518</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.007819207092366755</v>
+      </c>
+      <c r="K36" t="n">
+        <v>-0.8853590229606662</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.9353369576939384</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.7506249375062494</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0.5024497550244975</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Female_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>16</v>
+      </c>
+      <c r="F37" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2.177530382264464</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1.448046302578601</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.7294840796858637</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.003218863510540653</v>
+      </c>
+      <c r="K37" t="n">
+        <v>-0.4929698689218412</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.6339726603533002</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.0147985201479852</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0.0154984501549845</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Female_5-40_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>238</v>
+      </c>
+      <c r="F38" t="n">
+        <v>7788</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2.464836462532876</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-0.008569098016178771</v>
+      </c>
+      <c r="I38" t="n">
+        <v>2.473405560549054</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.0001299447870246792</v>
+      </c>
+      <c r="K38" t="n">
+        <v>-0.5271075107304388</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.5218284025415864</v>
+      </c>
+      <c r="M38" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N38" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Male_40-90_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>40-90</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>238</v>
+      </c>
+      <c r="F39" t="n">
+        <v>7788</v>
+      </c>
+      <c r="G39" t="n">
+        <v>3.924168775186589</v>
+      </c>
+      <c r="H39" t="n">
+        <v>3.229780626449666</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.6943881487369232</v>
+      </c>
+      <c r="J39" t="n">
+        <v>-0.001008698892644864</v>
+      </c>
+      <c r="K39" t="n">
+        <v>-0.3105360653635225</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.3300621018083453</v>
+      </c>
+      <c r="M39" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N39" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Male_40-90_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>21</v>
+      </c>
+      <c r="F40" t="n">
+        <v>7541</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.06202825830603671</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-0.003283886222118988</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.0653121445281557</v>
+      </c>
+      <c r="J40" t="n">
+        <v>-0.001502836148000746</v>
+      </c>
+      <c r="K40" t="n">
+        <v>-0.8191085024433405</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.8020183434341948</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.4357564243575642</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0.8720127987201279</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Male_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>21</v>
+      </c>
+      <c r="F41" t="n">
+        <v>7541</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2.707086686322044</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1.496159184830526</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1.210927501491518</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.000626681653298123</v>
+      </c>
+      <c r="K41" t="n">
+        <v>-0.4407941709759279</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.5566397795006385</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.0003999600039996001</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0.0003999600039996001</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/South Asian/South Asian_Male_5-40_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Turkish</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>268</v>
+      </c>
+      <c r="F42" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-0.4677516761140262</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-0.008381465306172826</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-0.4593702108078534</v>
+      </c>
+      <c r="J42" t="n">
+        <v>-0.0001816392540933913</v>
+      </c>
+      <c r="K42" t="n">
+        <v>-0.2337374798071015</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.2313211769159541</v>
+      </c>
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.0001999800019998</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Turkish/Turkish_Female_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>268</v>
+      </c>
+      <c r="F43" t="n">
+        <v>8505</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2.414725820022386</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.448046302578601</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.966679517443785</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.0006014017855444011</v>
+      </c>
+      <c r="K43" t="n">
+        <v>-0.137982053731996</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.1481828379357412</v>
+      </c>
+      <c r="M43" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N43" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Turkish/Turkish_Female_5-40_MAE_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>5-40</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
         <v>154</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F44" t="n">
         <v>7541</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G44" t="n">
+        <v>-0.2471475670944699</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-0.003283886222118988</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-0.2438636808723509</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.002201119318941359</v>
+      </c>
+      <c r="K44" t="n">
+        <v>-0.3083814391817878</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.3067473852108863</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.9394060593940606</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0.1230876912308769</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Turkish/Turkish_Male_5-40_BAG_permutation_histogram.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>5-40</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>154</v>
+      </c>
+      <c r="F45" t="n">
+        <v>7541</v>
+      </c>
+      <c r="G45" t="n">
         <v>2.709167943982263</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H45" t="n">
         <v>1.496159184830526</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I45" t="n">
         <v>1.213008759151737</v>
       </c>
-      <c r="I19" t="n">
-        <v>-0.0002645685282695053</v>
-      </c>
-      <c r="J19" t="n">
-        <v>-0.1821763935861646</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.1928000122279795</v>
-      </c>
-      <c r="L19" t="n">
-        <v>9.999000099990002e-05</v>
-      </c>
-      <c r="M19" t="n">
-        <v>9.999000099990002e-05</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Turkish/Turkish_Male_5-40_permutation_histogram.png</t>
+      <c r="J45" t="n">
+        <v>-0.0006427532796438819</v>
+      </c>
+      <c r="K45" t="n">
+        <v>-0.1845854719708071</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.1962131529597672</v>
+      </c>
+      <c r="M45" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="N45" t="n">
+        <v>9.999000099990002e-05</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>/Users/andrewli/Documents/Frangou Lab/BrainAGE/CentileBrain_BrainAGE/analyses/brainage_gap/outputs/permutation/Plots/Turkish/Turkish_Male_5-40_MAE_permutation_histogram.png</t>
         </is>
       </c>
     </row>

</xml_diff>